<commit_message>
feat: checkpoint experiment workflow and department data
</commit_message>
<xml_diff>
--- a/tasks/export-002-screenshots/selected-projects.xlsx
+++ b/tasks/export-002-screenshots/selected-projects.xlsx
@@ -75,10 +75,10 @@
     <x:t>통화</x:t>
   </x:si>
   <x:si>
-    <x:t>SEL-B-1784365054363</x:t>
-  </x:si>
-  <x:si>
-    <x:t>합성 선택 프로젝트 B 1784365054363</x:t>
+    <x:t>SEL-B-1784462644155</x:t>
+  </x:si>
+  <x:si>
+    <x:t>합성 선택 프로젝트 B 1784462644155</x:t>
   </x:si>
   <x:si>
     <x:t>Synthetic Selected Export Customer</x:t>
@@ -108,10 +108,10 @@
     <x:t>KRW</x:t>
   </x:si>
   <x:si>
-    <x:t>SEL-A-1784365054363</x:t>
-  </x:si>
-  <x:si>
-    <x:t>합성 선택 프로젝트 A 1784365054363</x:t>
+    <x:t>SEL-A-1784462644155</x:t>
+  </x:si>
+  <x:si>
+    <x:t>합성 선택 프로젝트 A 1784462644155</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -804,7 +804,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="2">
-        <x:v>46221.3733255556</x:v>
+        <x:v>46222.502835787</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:15">

</xml_diff>